<commit_message>
Update analysis, charts and scripts
</commit_message>
<xml_diff>
--- a/msa_map/data/analysis/MSA_Indicator_Tracker.xlsx
+++ b/msa_map/data/analysis/MSA_Indicator_Tracker.xlsx
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="£#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -294,7 +295,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -597,6 +598,27 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -966,7 +988,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="77" min="1" max="1"/>
     <col width="22" customWidth="1" style="77" min="2" max="2"/>
@@ -3122,7 +3144,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="77" min="1" max="1"/>
     <col width="22" customWidth="1" style="77" min="2" max="2"/>
@@ -4558,32 +4580,45 @@
           <t>IMD 2025 average rank</t>
         </is>
       </c>
-      <c r="D30" s="40" t="n"/>
-      <c r="E30" s="39" t="inlineStr">
-        <is>
-          <t>rank</t>
-        </is>
-      </c>
-      <c r="F30" s="39" t="inlineStr">
+      <c r="D30" s="104" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="98" t="inlineStr">
+        <is>
+          <t>% LSOAs</t>
+        </is>
+      </c>
+      <c r="F30" s="98" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G30" s="39" t="n"/>
-      <c r="H30" s="36" t="n"/>
-      <c r="I30" s="36" t="n"/>
+      <c r="G30" s="104" t="n">
+        <v>10</v>
+      </c>
+      <c r="H30" s="105">
+        <f>D30-G30</f>
+        <v/>
+      </c>
+      <c r="I30" s="99" t="inlineStr">
+        <is>
+          <t>Higher = more deprived</t>
+        </is>
+      </c>
       <c r="J30" s="39" t="n"/>
       <c r="K30" s="36" t="n"/>
       <c r="L30" s="39" t="n"/>
-      <c r="M30" s="39" t="n"/>
-      <c r="N30" s="41" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-      <c r="O30" s="39" t="inlineStr">
-        <is>
-          <t>MHCLG IMD 2025 File 10</t>
+      <c r="M30" s="100" t="n">
+        <v>20</v>
+      </c>
+      <c r="N30" s="86" t="inlineStr">
+        <is>
+          <t>Populated</t>
+        </is>
+      </c>
+      <c r="O30" s="98" t="inlineStr">
+        <is>
+          <t>IMD 2025. % of 500 LSOAs in YNYCA falling in most deprived 10% nationally. England benchmark = 10.0% by definition. YNYCA rank 20/20 — least deprived MSA. Decile distribution heavily skewed toward less deprived end (median rank 21,730 vs England 16,878).</t>
         </is>
       </c>
     </row>
@@ -4603,32 +4638,43 @@
           <t>% LSOAs in most deprived 10%</t>
         </is>
       </c>
-      <c r="D31" s="40" t="n"/>
-      <c r="E31" s="39" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="F31" s="39" t="inlineStr">
+      <c r="D31" s="106" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E31" s="98" t="inlineStr">
+        <is>
+          <t>% LSOAs</t>
+        </is>
+      </c>
+      <c r="F31" s="98" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G31" s="39" t="n"/>
-      <c r="H31" s="36" t="n"/>
-      <c r="I31" s="36" t="n"/>
+      <c r="G31" s="106" t="n">
+        <v>20</v>
+      </c>
+      <c r="H31" s="107">
+        <f>D31-G31</f>
+        <v/>
+      </c>
+      <c r="I31" s="99" t="inlineStr">
+        <is>
+          <t>Higher = more deprived</t>
+        </is>
+      </c>
       <c r="J31" s="39" t="n"/>
       <c r="K31" s="36" t="n"/>
       <c r="L31" s="39" t="n"/>
       <c r="M31" s="39" t="n"/>
-      <c r="N31" s="41" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-      <c r="O31" s="39" t="inlineStr">
-        <is>
-          <t>MHCLG IMD 2025 File 10</t>
+      <c r="N31" s="86" t="inlineStr">
+        <is>
+          <t>Populated</t>
+        </is>
+      </c>
+      <c r="O31" s="98" t="inlineStr">
+        <is>
+          <t>IMD 2025. % of LSOAs in deciles 1 or 2 (most deprived 20% nationally). England benchmark = 20.0% by definition. YNYCA 6.2% — well below benchmark, consistent with rural affluent character. Avg IMD rank 21,081 vs England avg 16,878.</t>
         </is>
       </c>
     </row>
@@ -4739,7 +4785,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="77" min="1" max="1"/>
     <col width="38" customWidth="1" style="77" min="2" max="2"/>
@@ -5617,64 +5663,146 @@
         </is>
       </c>
       <c r="D19" s="51" t="n"/>
-      <c r="E19" s="50" t="n"/>
-      <c r="F19" s="50" t="n"/>
-      <c r="G19" s="50" t="n"/>
-      <c r="H19" s="50" t="n"/>
-      <c r="I19" s="50" t="n"/>
-      <c r="J19" s="50" t="n"/>
-      <c r="K19" s="50" t="n"/>
-      <c r="L19" s="50" t="n"/>
-      <c r="M19" s="50" t="n"/>
-      <c r="N19" s="52" t="n"/>
-      <c r="O19" s="50" t="n"/>
-      <c r="P19" s="50" t="n"/>
-      <c r="Q19" s="50" t="n"/>
-      <c r="R19" s="50" t="n"/>
-      <c r="S19" s="50" t="n"/>
-      <c r="T19" s="50" t="n"/>
-      <c r="U19" s="50" t="n"/>
-      <c r="V19" s="50" t="n"/>
-      <c r="W19" s="50" t="n"/>
-      <c r="X19" s="50" t="n"/>
+      <c r="E19" s="91" t="n">
+        <v>23</v>
+      </c>
+      <c r="F19" s="91" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="G19" s="108" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H19" s="91" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="I19" s="91" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J19" s="108" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="K19" s="108" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="L19" s="108" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="M19" s="91" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="N19" s="86" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" s="108" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="P19" s="108" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="Q19" s="108" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="R19" s="86" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="S19" s="86" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="T19" s="86" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U19" s="108" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="V19" s="108" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="W19" s="86" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="X19" s="108" t="n">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1" s="77">
       <c r="A20" s="53" t="inlineStr">
         <is>
-          <t>SAFETY_001</t>
+          <t>IMD_002</t>
         </is>
       </c>
       <c r="B20" s="54" t="inlineStr">
         <is>
-          <t>Notifiable offences</t>
+          <t>% LSOAs in most deprived 20%</t>
         </is>
       </c>
       <c r="C20" s="55" t="inlineStr">
         <is>
-          <t>per 1,000</t>
-        </is>
-      </c>
-      <c r="D20" s="51" t="n"/>
-      <c r="E20" s="55" t="n"/>
-      <c r="F20" s="55" t="n"/>
-      <c r="G20" s="55" t="n"/>
-      <c r="H20" s="55" t="n"/>
-      <c r="I20" s="55" t="n"/>
-      <c r="J20" s="55" t="n"/>
-      <c r="K20" s="55" t="n"/>
-      <c r="L20" s="55" t="n"/>
-      <c r="M20" s="55" t="n"/>
-      <c r="N20" s="52" t="n"/>
-      <c r="O20" s="55" t="n"/>
-      <c r="P20" s="55" t="n"/>
-      <c r="Q20" s="55" t="n"/>
-      <c r="R20" s="55" t="n"/>
-      <c r="S20" s="55" t="n"/>
-      <c r="T20" s="55" t="n"/>
-      <c r="U20" s="55" t="n"/>
-      <c r="V20" s="55" t="n"/>
-      <c r="W20" s="55" t="n"/>
-      <c r="X20" s="55" t="n"/>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>20</v>
+      </c>
+      <c r="E20" s="109" t="n">
+        <v>37</v>
+      </c>
+      <c r="F20" s="109" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="G20" s="109" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="H20" s="109" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="I20" s="109" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="J20" s="109" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="K20" s="109" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="L20" s="109" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="M20" s="109" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="N20" s="110" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="O20" s="109" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="P20" s="109" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="Q20" s="109" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="R20" s="109" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="S20" s="109" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T20" s="109" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="U20" s="109" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="V20" s="109" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="W20" s="109" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="X20" s="109" t="n">
+        <v>12.6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5771,7 +5899,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="77" min="1" max="1"/>
     <col width="38" customWidth="1" style="77" min="2" max="2"/>
@@ -6136,7 +6264,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" style="77" min="1" max="1"/>
     <col width="18" customWidth="1" style="77" min="2" max="2"/>

</xml_diff>